<commit_message>
Aggiornate tariffe E.ON luglio 2026: valori residenziali EE da PDF, business e microbusiness gas allineati
</commit_message>
<xml_diff>
--- a/estrazioni_tariffe/eon_tariffe_2026-07.xlsx
+++ b/estrazioni_tariffe/eon_tariffe_2026-07.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,21 +27,13 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9EAF7"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -56,9 +48,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -425,92 +416,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="74" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
-    <col width="52" customWidth="1" min="14" max="14"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>provider</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>segmento</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>commodity</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>offer_type</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>offer_name</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>valid_from</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>valid_to</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>component</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>uom</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>index_name</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>codice_offerta</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>source_pdf</t>
         </is>
@@ -542,10 +517,10 @@
           <t>E.ON Flex Gas</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H2" t="inlineStr">
@@ -608,10 +583,10 @@
           <t>E.ON Flex Gas</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H3" t="inlineStr">
@@ -674,10 +649,10 @@
           <t>E.ON Flex Gas</t>
         </is>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H4" t="inlineStr">
@@ -740,10 +715,10 @@
           <t>E.ON Flex Gas Protetta</t>
         </is>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H5" t="inlineStr">
@@ -806,10 +781,10 @@
           <t>E.ON Flex Gas Protetta</t>
         </is>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H6" t="inlineStr">
@@ -872,10 +847,10 @@
           <t>E.ON Flex Gas Protetta</t>
         </is>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H7" t="inlineStr">
@@ -938,10 +913,10 @@
           <t>E.ON Gas Protetta Per 24</t>
         </is>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H8" t="inlineStr">
@@ -999,10 +974,10 @@
           <t>E.ON Gas Protetta Per 24</t>
         </is>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H9" t="inlineStr">
@@ -1060,10 +1035,10 @@
           <t>E.ON Gas Tua</t>
         </is>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G10" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H10" t="inlineStr">
@@ -1121,10 +1096,10 @@
           <t>E.ON Gas Tua</t>
         </is>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G11" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H11" t="inlineStr">
@@ -1182,10 +1157,10 @@
           <t>E.ON Gas Tua</t>
         </is>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="G12" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H12" t="inlineStr">
@@ -1243,10 +1218,10 @@
           <t>E.ON GasVerde Protetta</t>
         </is>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="G13" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H13" t="inlineStr">
@@ -1304,10 +1279,10 @@
           <t>E.ON GasVerde Protetta</t>
         </is>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G14" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H14" t="inlineStr">
@@ -1365,10 +1340,10 @@
           <t>E.ON Flex Luce</t>
         </is>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="F15" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G15" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H15" t="inlineStr">
@@ -1396,7 +1371,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZG36S0DFLX000C000</t>
+          <t>000362ESVFL01XXZG36T0DFLX000C000</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1431,10 +1406,10 @@
           <t>E.ON Flex Luce</t>
         </is>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G16" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H16" t="inlineStr">
@@ -1462,7 +1437,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZG36S0DFLX000C000</t>
+          <t>000362ESVFL01XXZG36T0DFLX000C000</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1497,10 +1472,10 @@
           <t>E.ON Flex Luce</t>
         </is>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="F17" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="G17" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H17" t="inlineStr">
@@ -1514,7 +1489,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>121.23</v>
+        <v>121.11</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1528,7 +1503,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZG36S0DFLX000C000</t>
+          <t>000362ESVFL01XXZG36T0DFLX000C000</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1563,10 +1538,10 @@
           <t>E.ON Flex Luce</t>
         </is>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="F18" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="G18" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H18" t="inlineStr">
@@ -1594,7 +1569,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZG36S0DFLX000C000</t>
+          <t>000362ESVFL01XXZG36T0DFLX000C000</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1629,10 +1604,10 @@
           <t>E.ON Flex Luce Casa</t>
         </is>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="F19" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="G19" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H19" t="inlineStr">
@@ -1660,7 +1635,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZG36S0DACR000E000</t>
+          <t>000362ESVFL01XXZG36T0DACR000E000</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1695,10 +1670,10 @@
           <t>E.ON Flex Luce Casa</t>
         </is>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="F20" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="G20" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H20" t="inlineStr">
@@ -1726,7 +1701,7 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZG36S0DACR000E000</t>
+          <t>000362ESVFL01XXZG36T0DACR000E000</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1761,10 +1736,10 @@
           <t>E.ON Flex Luce Casa</t>
         </is>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="F21" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G21" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H21" t="inlineStr">
@@ -1778,7 +1753,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>145.23</v>
+        <v>145.11</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -1792,7 +1767,7 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZG36S0DACR000E000</t>
+          <t>000362ESVFL01XXZG36T0DACR000E000</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1827,10 +1802,10 @@
           <t>E.ON Flex Luce Casa</t>
         </is>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="F22" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G22" s="2" t="n">
+      <c r="G22" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H22" t="inlineStr">
@@ -1858,7 +1833,7 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZG36S0DACR000E000</t>
+          <t>000362ESVFL01XXZG36T0DACR000E000</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1893,10 +1868,10 @@
           <t>E.ON Flex Luce Per24</t>
         </is>
       </c>
-      <c r="F23" s="2" t="n">
+      <c r="F23" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G23" s="2" t="n">
+      <c r="G23" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H23" t="inlineStr">
@@ -1924,7 +1899,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZJ36S0DRI0000D000</t>
+          <t>000362ESVFL01XXZJ36T0DRI0000D000</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1959,10 +1934,10 @@
           <t>E.ON Flex Luce Per24</t>
         </is>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="F24" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G24" s="2" t="n">
+      <c r="G24" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H24" t="inlineStr">
@@ -1990,7 +1965,7 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZJ36S0DRI0000D000</t>
+          <t>000362ESVFL01XXZJ36T0DRI0000D000</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2025,10 +2000,10 @@
           <t>E.ON Flex Luce Per24</t>
         </is>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="F25" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G25" s="2" t="n">
+      <c r="G25" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H25" t="inlineStr">
@@ -2042,7 +2017,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>121.23</v>
+        <v>121.11</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -2056,7 +2031,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZJ36S0DRI0000D000</t>
+          <t>000362ESVFL01XXZJ36T0DRI0000D000</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -2091,10 +2066,10 @@
           <t>E.ON Flex Luce Per24</t>
         </is>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="F26" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G26" s="2" t="n">
+      <c r="G26" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H26" t="inlineStr">
@@ -2122,7 +2097,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>000362ESVFL01XXZJ36S0DRI0000D000</t>
+          <t>000362ESVFL01XXZJ36T0DRI0000D000</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -2157,10 +2132,10 @@
           <t>E.ON Ore Per Te</t>
         </is>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="F27" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G27" s="2" t="n">
+      <c r="G27" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H27" t="inlineStr">
@@ -2174,7 +2149,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>0.1254</v>
+        <v>0.1705</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -2183,7 +2158,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>000362ESFML01XXLZ16S0D000000A000</t>
+          <t>000362ESFML01XXLZ16T0D000000A000</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -2218,10 +2193,10 @@
           <t>E.ON Ore Per Te</t>
         </is>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="F28" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G28" s="2" t="n">
+      <c r="G28" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H28" t="inlineStr">
@@ -2235,7 +2210,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>121.23</v>
+        <v>121.11</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -2244,7 +2219,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>000362ESFML01XXLZ16S0D000000A000</t>
+          <t>000362ESFML01XXLZ16T0D000000A000</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2279,10 +2254,10 @@
           <t>E.ON Luce Casa Per 24</t>
         </is>
       </c>
-      <c r="F29" s="2" t="n">
+      <c r="F29" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G29" s="2" t="n">
+      <c r="G29" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H29" t="inlineStr">
@@ -2296,7 +2271,7 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>0.1398</v>
+        <v>0.1343</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -2305,7 +2280,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>000362ESFML01XXZL16S0DACR000C000</t>
+          <t>000362ESFML01XXZL16T0DACR000C000</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2340,10 +2315,10 @@
           <t>E.ON Luce Casa Per 24</t>
         </is>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="F30" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G30" s="2" t="n">
+      <c r="G30" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H30" t="inlineStr">
@@ -2357,7 +2332,7 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>0.145</v>
+        <v>0.1384</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -2366,7 +2341,7 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>000362ESFML01XXZL16S0DACR000C000</t>
+          <t>000362ESFML01XXZL16T0DACR000C000</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2401,10 +2376,10 @@
           <t>E.ON Luce Casa Per 24</t>
         </is>
       </c>
-      <c r="F31" s="2" t="n">
+      <c r="F31" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G31" s="2" t="n">
+      <c r="G31" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H31" t="inlineStr">
@@ -2418,7 +2393,7 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>0.1372</v>
+        <v>0.1318</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -2427,7 +2402,7 @@
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>000362ESFML01XXZL16S0DACR000C000</t>
+          <t>000362ESFML01XXZL16T0DACR000C000</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2462,10 +2437,10 @@
           <t>E.ON Luce Casa Per 24</t>
         </is>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="F32" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G32" s="2" t="n">
+      <c r="G32" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H32" t="inlineStr">
@@ -2479,7 +2454,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>145.23</v>
+        <v>145.11</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -2488,7 +2463,7 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>000362ESFML01XXZL16S0DACR000C000</t>
+          <t>000362ESFML01XXZL16T0DACR000C000</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2523,10 +2498,10 @@
           <t>E.ON Luce Tua Per 24</t>
         </is>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="F33" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G33" s="2" t="n">
+      <c r="G33" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H33" t="inlineStr">
@@ -2540,7 +2515,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>0.1503</v>
+        <v>0.1448</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -2549,7 +2524,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>000362ESFML01XXZL16S0D000000B000</t>
+          <t>000362ESFML01XXZL16T0D000000B000</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2584,10 +2559,10 @@
           <t>E.ON Luce Tua Per 24</t>
         </is>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="F34" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G34" s="2" t="n">
+      <c r="G34" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H34" t="inlineStr">
@@ -2601,7 +2576,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>0.1544</v>
+        <v>0.1488</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -2610,7 +2585,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>000362ESFML01XXZL16S0D000000B000</t>
+          <t>000362ESFML01XXZL16T0D000000B000</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2645,10 +2620,10 @@
           <t>E.ON Luce Tua Per 24</t>
         </is>
       </c>
-      <c r="F35" s="2" t="n">
+      <c r="F35" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G35" s="2" t="n">
+      <c r="G35" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H35" t="inlineStr">
@@ -2662,7 +2637,7 @@
         </is>
       </c>
       <c r="J35" t="n">
-        <v>0.1476</v>
+        <v>0.1423</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -2671,7 +2646,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>000362ESFML01XXZL16S0D000000B000</t>
+          <t>000362ESFML01XXZL16T0D000000B000</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2706,10 +2681,10 @@
           <t>E.ON Luce Tua Per 24</t>
         </is>
       </c>
-      <c r="F36" s="2" t="n">
+      <c r="F36" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G36" s="2" t="n">
+      <c r="G36" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H36" t="inlineStr">
@@ -2723,7 +2698,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>121.23</v>
+        <v>121.11</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -2732,7 +2707,7 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>000362ESFML01XXZL16S0D000000B000</t>
+          <t>000362ESFML01XXZL16T0D000000B000</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2767,10 +2742,10 @@
           <t>E.ON Luce Tua Per 24</t>
         </is>
       </c>
-      <c r="F37" s="2" t="n">
+      <c r="F37" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G37" s="2" t="n">
+      <c r="G37" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H37" t="inlineStr">
@@ -2793,7 +2768,7 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>000362ESFML01XXZL16S0D000000B000</t>
+          <t>000362ESFML01XXZL16T0D000000B000</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2828,10 +2803,10 @@
           <t>E.ON LuceVerde Casa</t>
         </is>
       </c>
-      <c r="F38" s="2" t="n">
+      <c r="F38" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G38" s="2" t="n">
+      <c r="G38" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H38" t="inlineStr">
@@ -2845,7 +2820,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>0.1665</v>
+        <v>0.1539</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -2854,7 +2829,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>000362ESFML01XXLS16S0DACR000E000</t>
+          <t>000362ESFML01XXLS16T0DACR000E000</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2889,10 +2864,10 @@
           <t>E.ON LuceVerde Casa</t>
         </is>
       </c>
-      <c r="F39" s="2" t="n">
+      <c r="F39" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G39" s="2" t="n">
+      <c r="G39" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H39" t="inlineStr">
@@ -2906,7 +2881,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>0.1691</v>
+        <v>0.1567</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -2915,7 +2890,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>000362ESFML01XXLS16S0DACR000E000</t>
+          <t>000362ESFML01XXLS16T0DACR000E000</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2950,10 +2925,10 @@
           <t>E.ON LuceVerde Casa</t>
         </is>
       </c>
-      <c r="F40" s="2" t="n">
+      <c r="F40" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G40" s="2" t="n">
+      <c r="G40" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H40" t="inlineStr">
@@ -2967,7 +2942,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>0.165</v>
+        <v>0.1521</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -2976,7 +2951,7 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>000362ESFML01XXLS16S0DACR000E000</t>
+          <t>000362ESFML01XXLS16T0DACR000E000</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -3011,10 +2986,10 @@
           <t>E.ON LuceVerde Casa</t>
         </is>
       </c>
-      <c r="F41" s="2" t="n">
+      <c r="F41" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G41" s="2" t="n">
+      <c r="G41" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H41" t="inlineStr">
@@ -3028,7 +3003,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>145.23</v>
+        <v>145.11</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -3037,7 +3012,7 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>000362ESFML01XXLS16S0DACR000E000</t>
+          <t>000362ESFML01XXLS16T0DACR000E000</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -3072,10 +3047,10 @@
           <t>E.ON Luce Tua</t>
         </is>
       </c>
-      <c r="F42" s="2" t="n">
+      <c r="F42" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G42" s="2" t="n">
+      <c r="G42" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H42" t="inlineStr">
@@ -3089,7 +3064,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>0.1514</v>
+        <v>0.1387</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -3098,7 +3073,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>000362ESFML01XXLS16S0D000000A000</t>
+          <t>000362ESFML01XXLS16T0D000000A000</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -3133,10 +3108,10 @@
           <t>E.ON Luce Tua</t>
         </is>
       </c>
-      <c r="F43" s="2" t="n">
+      <c r="F43" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G43" s="2" t="n">
+      <c r="G43" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H43" t="inlineStr">
@@ -3150,7 +3125,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>0.154</v>
+        <v>0.1415</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -3159,7 +3134,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>000362ESFML01XXLS16S0D000000A000</t>
+          <t>000362ESFML01XXLS16T0D000000A000</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -3194,10 +3169,10 @@
           <t>E.ON Luce Tua</t>
         </is>
       </c>
-      <c r="F44" s="2" t="n">
+      <c r="F44" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G44" s="2" t="n">
+      <c r="G44" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H44" t="inlineStr">
@@ -3211,7 +3186,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>0.1498</v>
+        <v>0.137</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -3220,7 +3195,7 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>000362ESFML01XXLS16S0D000000A000</t>
+          <t>000362ESFML01XXLS16T0D000000A000</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3255,10 +3230,10 @@
           <t>E.ON Luce Tua</t>
         </is>
       </c>
-      <c r="F45" s="2" t="n">
+      <c r="F45" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G45" s="2" t="n">
+      <c r="G45" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H45" t="inlineStr">
@@ -3272,7 +3247,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>121.23</v>
+        <v>121.11</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -3281,7 +3256,7 @@
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>000362ESFML01XXLS16S0D000000A000</t>
+          <t>000362ESFML01XXLS16T0D000000A000</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3316,10 +3291,10 @@
           <t>E.ON Luce Tua</t>
         </is>
       </c>
-      <c r="F46" s="2" t="n">
+      <c r="F46" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G46" s="2" t="n">
+      <c r="G46" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H46" t="inlineStr">
@@ -3342,7 +3317,7 @@
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>000362ESFML01XXLS16S0D000000A000</t>
+          <t>000362ESFML01XXLS16T0D000000A000</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3377,10 +3352,10 @@
           <t>E.ON Gas Impresa CLSC</t>
         </is>
       </c>
-      <c r="F47" s="2" t="n">
+      <c r="F47" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G47" s="2" t="n">
+      <c r="G47" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H47" t="inlineStr">
@@ -3443,10 +3418,10 @@
           <t>E.ON Gas Impresa CLSC</t>
         </is>
       </c>
-      <c r="F48" s="2" t="n">
+      <c r="F48" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G48" s="2" t="n">
+      <c r="G48" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H48" t="inlineStr">
@@ -3509,10 +3484,10 @@
           <t>E.ON Gas Impresa CLSC</t>
         </is>
       </c>
-      <c r="F49" s="2" t="n">
+      <c r="F49" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G49" s="2" t="n">
+      <c r="G49" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H49" t="inlineStr">
@@ -3575,10 +3550,10 @@
           <t>E.ON Gas Impresa CLSC</t>
         </is>
       </c>
-      <c r="F50" s="2" t="n">
+      <c r="F50" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G50" s="2" t="n">
+      <c r="G50" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H50" t="inlineStr">
@@ -3641,10 +3616,10 @@
           <t>E.ON Gas Impresa CLSE</t>
         </is>
       </c>
-      <c r="F51" s="2" t="n">
+      <c r="F51" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G51" s="2" t="n">
+      <c r="G51" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H51" t="inlineStr">
@@ -3707,10 +3682,10 @@
           <t>E.ON Gas Impresa CLSE</t>
         </is>
       </c>
-      <c r="F52" s="2" t="n">
+      <c r="F52" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G52" s="2" t="n">
+      <c r="G52" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H52" t="inlineStr">
@@ -3773,10 +3748,10 @@
           <t>E.ON Gas Impresa CLSE</t>
         </is>
       </c>
-      <c r="F53" s="2" t="n">
+      <c r="F53" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G53" s="2" t="n">
+      <c r="G53" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H53" t="inlineStr">
@@ -3839,10 +3814,10 @@
           <t>E.ON Gas Impresa CLSE</t>
         </is>
       </c>
-      <c r="F54" s="2" t="n">
+      <c r="F54" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G54" s="2" t="n">
+      <c r="G54" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H54" t="inlineStr">
@@ -3905,10 +3880,10 @@
           <t>E.ON ChiaraGas Rinnovo CLSC</t>
         </is>
       </c>
-      <c r="F55" s="2" t="n">
+      <c r="F55" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G55" s="2" t="n">
+      <c r="G55" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H55" t="inlineStr">
@@ -3966,10 +3941,10 @@
           <t>E.ON ChiaraGas Rinnovo CLSC</t>
         </is>
       </c>
-      <c r="F56" s="2" t="n">
+      <c r="F56" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G56" s="2" t="n">
+      <c r="G56" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H56" t="inlineStr">
@@ -4027,10 +4002,10 @@
           <t>E.ON ChiaraGas Rinnovo CLSC</t>
         </is>
       </c>
-      <c r="F57" s="2" t="n">
+      <c r="F57" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G57" s="2" t="n">
+      <c r="G57" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H57" t="inlineStr">
@@ -4088,10 +4063,10 @@
           <t>E.ON ChiaraGas Rinnovo CLSE</t>
         </is>
       </c>
-      <c r="F58" s="2" t="n">
+      <c r="F58" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G58" s="2" t="n">
+      <c r="G58" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H58" t="inlineStr">
@@ -4149,10 +4124,10 @@
           <t>E.ON ChiaraGas Rinnovo CLSE</t>
         </is>
       </c>
-      <c r="F59" s="2" t="n">
+      <c r="F59" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G59" s="2" t="n">
+      <c r="G59" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H59" t="inlineStr">
@@ -4210,10 +4185,10 @@
           <t>E.ON ChiaraGas Rinnovo CLSE</t>
         </is>
       </c>
-      <c r="F60" s="2" t="n">
+      <c r="F60" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G60" s="2" t="n">
+      <c r="G60" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H60" t="inlineStr">
@@ -4271,10 +4246,10 @@
           <t>E.ON LuceDinamica ECO CLSC</t>
         </is>
       </c>
-      <c r="F61" s="2" t="n">
+      <c r="F61" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="G61" s="2" t="n">
+      <c r="G61" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="H61" t="inlineStr">
@@ -4337,10 +4312,10 @@
           <t>E.ON LuceDinamica ECO CLSC</t>
         </is>
       </c>
-      <c r="F62" s="2" t="n">
+      <c r="F62" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="G62" s="2" t="n">
+      <c r="G62" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="H62" t="inlineStr">
@@ -4403,10 +4378,10 @@
           <t>E.ON LuceDinamica ECO CLSC</t>
         </is>
       </c>
-      <c r="F63" s="2" t="n">
+      <c r="F63" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="G63" s="2" t="n">
+      <c r="G63" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="H63" t="inlineStr">
@@ -4469,10 +4444,10 @@
           <t>E.ON LuceDinamica ECO CLSE</t>
         </is>
       </c>
-      <c r="F64" s="2" t="n">
+      <c r="F64" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="G64" s="2" t="n">
+      <c r="G64" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="H64" t="inlineStr">
@@ -4535,10 +4510,10 @@
           <t>E.ON LuceDinamica ECO CLSE</t>
         </is>
       </c>
-      <c r="F65" s="2" t="n">
+      <c r="F65" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="G65" s="2" t="n">
+      <c r="G65" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="H65" t="inlineStr">
@@ -4601,10 +4576,10 @@
           <t>E.ON LuceDinamica ECO CLSE</t>
         </is>
       </c>
-      <c r="F66" s="2" t="n">
+      <c r="F66" s="1" t="n">
         <v>46191</v>
       </c>
-      <c r="G66" s="2" t="n">
+      <c r="G66" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="H66" t="inlineStr">
@@ -4667,10 +4642,10 @@
           <t>E.ON EnergiaChiara ECO CLSC</t>
         </is>
       </c>
-      <c r="F67" s="2" t="n">
+      <c r="F67" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G67" s="2" t="n">
+      <c r="G67" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H67" t="inlineStr">
@@ -4728,10 +4703,10 @@
           <t>E.ON EnergiaChiara ECO CLSC</t>
         </is>
       </c>
-      <c r="F68" s="2" t="n">
+      <c r="F68" s="1" t="n">
         <v>46204</v>
       </c>
-      <c r="G68" s="2" t="n">
+      <c r="G68" s="1" t="n">
         <v>46234</v>
       </c>
       <c r="H68" t="inlineStr">
@@ -4789,10 +4764,10 @@
           <t>E.ON EnergiaChiara ECO CLSE</t>
         </is>
       </c>
-      <c r="F69" s="2" t="n">
+      <c r="F69" s="1" t="n">
         <v>46206</v>
       </c>
-      <c r="G69" s="2" t="n">
+      <c r="G69" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="H69" t="inlineStr">
@@ -4850,10 +4825,10 @@
           <t>E.ON EnergiaChiara ECO CLSE</t>
         </is>
       </c>
-      <c r="F70" s="2" t="n">
+      <c r="F70" s="1" t="n">
         <v>46206</v>
       </c>
-      <c r="G70" s="2" t="n">
+      <c r="G70" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="H70" t="inlineStr">
@@ -4911,10 +4886,10 @@
           <t>E.ON EnergiaChiara ECO CLSE</t>
         </is>
       </c>
-      <c r="F71" s="2" t="n">
+      <c r="F71" s="1" t="n">
         <v>46206</v>
       </c>
-      <c r="G71" s="2" t="n">
+      <c r="G71" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="H71" t="inlineStr">
@@ -4972,10 +4947,10 @@
           <t>E.ON EnergiaChiara ECO CLSE</t>
         </is>
       </c>
-      <c r="F72" s="2" t="n">
+      <c r="F72" s="1" t="n">
         <v>46206</v>
       </c>
-      <c r="G72" s="2" t="n">
+      <c r="G72" s="1" t="n">
         <v>46225</v>
       </c>
       <c r="H72" t="inlineStr">
@@ -4989,7 +4964,7 @@
         </is>
       </c>
       <c r="J72" t="n">
-        <v>192.71</v>
+        <v>142.71</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -5004,6 +4979,1821 @@
       <c r="N72" t="inlineStr">
         <is>
           <t>E.ON EnergiaChiara - ECO_6R.2_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSC</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>gestione_energetica</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J73" t="n">
+        <v>50</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Corrispettivo gestione energetica E.ON.</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000C000</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSE</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>gestione_energetica</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>50</v>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Corrispettivo gestione energetica E.ON.</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000E000</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSC</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>gestione_energetica</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J75" t="n">
+        <v>50</v>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Corrispettivo gestione energetica E.ON.</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000C000</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSC</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>bilanciamento</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Oneri integrativi di vendita E.ON.</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000C000</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSE</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>gestione_energetica</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
+        <v>50</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Corrispettivo gestione energetica E.ON.</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000E000</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>BUSINESS</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSE</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>bilanciamento</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Oneri integrativi di vendita E.ON.</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000E000</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSC</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>fee_energia</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>0.0837</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Omega su PSV DA.</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000C000</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSC</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>ccv_quota_fissa</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>143.64</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Quota fissa annua; per microbusiness include anche gestione energetica fissa.</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000C000</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSC</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>ccv_quota_variabile</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Commercializzazione al dettaglio quota variabile.</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000C000</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSC</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>bilanciamento</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Oneri integrativi di vendita E.ON.</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000C000</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSC</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>gestione_energetica</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J83" t="n">
+        <v>50</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Corrispettivo gestione energetica E.ON.</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000C000</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSE</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>fee_energia</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J84" t="n">
+        <v>0.1328</v>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>Omega su PSV DA.</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000E000</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSE</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>ccv_quota_fissa</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>143.64</v>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>Quota fissa annua; per microbusiness include anche gestione energetica fissa.</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000E000</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSE</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>ccv_quota_variabile</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J86" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>Commercializzazione al dettaglio quota variabile.</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000E000</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSE</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>bilanciamento</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J87" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>Oneri integrativi di vendita E.ON.</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000E000</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>VARIABILE</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa CLSE</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>gestione_energetica</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>50</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Corrispettivo gestione energetica E.ON.</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>000362GSVML01XXPX06S0M000000E000</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>E.ON Gas Impresa_6S_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSC</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>prezzo_fisso</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>Materia Prima Gas fissa.</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000C000</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSC</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>ccv_quota_fissa</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>143.64</v>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Quota fissa annua; per microbusiness include anche gestione energetica fissa.</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000C000</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSC</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>ccv_quota_variabile</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>Commercializzazione al dettaglio quota variabile.</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000C000</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSC</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>bilanciamento</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Oneri integrativi di vendita E.ON.</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000C000</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSC</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>gestione_energetica</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
+        <v>50</v>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>Corrispettivo gestione energetica E.ON.</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000C000</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSC.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSE</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>prezzo_fisso</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Materia Prima Gas fissa.</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000E000</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSE</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>ccv_quota_fissa</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J95" t="n">
+        <v>143.64</v>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Quota fissa annua; per microbusiness include anche gestione energetica fissa.</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000E000</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSE</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>ccv_quota_variabile</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J96" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>Commercializzazione al dettaglio quota variabile.</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000E000</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSE</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>bilanciamento</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>€/Smc</t>
+        </is>
+      </c>
+      <c r="J97" t="n">
+        <v>0.0095</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>PSV</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Oneri integrativi di vendita E.ON.</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000E000</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>GAS</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo CLSE</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>gestione_energetica</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J98" t="n">
+        <v>50</v>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Corrispettivo gestione energetica E.ON.</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>000362GSFML01XXYS06S4M000000E000</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>E.ON ChiaraGas Rinnovo_6S.4_M_CLSE.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>E.ON</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>MICROBUSINESS</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>EE</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>FISSA</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>E.ON EnergiaChiara ECO CLSE</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>gestione_energetica</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>€/anno</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>50</v>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>Corrispettivo gestione energetica E.ON.</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>000362ESFML01XXLS16S4M000000E000</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>E.ON EnergiaChiara - ECO_6S.4_M_CLSE.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>